<commit_message>
CORS und Environment Variables #257
</commit_message>
<xml_diff>
--- a/DAGoPERT_AILV.xlsx
+++ b/DAGoPERT_AILV.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr codeName="DieseArbeitsmappe" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Elena\Desktop\FH\INNO\AILV-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19F1B624-EE21-4850-B8C4-00423438D11B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75581E5C-1CF3-4858-84EF-48E6C2E81B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="758" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="636" yWindow="3360" windowWidth="22404" windowHeight="8880" tabRatio="758" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="18" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="172">
   <si>
     <t>Umsetzung</t>
   </si>
@@ -512,9 +512,6 @@
   </si>
   <si>
     <t>1.5</t>
-  </si>
-  <si>
-    <t>Aufgrund der fehlenden Erfahrung, wird die Schätzung vorerst ausgelassen</t>
   </si>
   <si>
     <t>2.1</t>
@@ -1843,49 +1840,49 @@
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>1.4828622159501934</c:v>
+                  <c:v>1.5448548269923559</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.5074068182081237</c:v>
+                  <c:v>1.5695820892751076</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.51695194130843</c:v>
+                  <c:v>1.5791982468295112</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.5224062973657477</c:v>
+                  <c:v>1.5846931940034561</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.528201550676648</c:v>
+                  <c:v>1.5905315753757725</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.5333150094803836</c:v>
+                  <c:v>1.5956830883513455</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.5425192353271073</c:v>
+                  <c:v>1.6049558117073777</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.5510416666666667</c:v>
+                  <c:v>1.6135416666666664</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.5595640980062258</c:v>
+                  <c:v>1.6221275216259552</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.5687683238529497</c:v>
+                  <c:v>1.6314002449819871</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.5738817826566851</c:v>
+                  <c:v>1.6365517579575606</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.5796770359675854</c:v>
+                  <c:v>1.642390139329877</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.5851313920249033</c:v>
+                  <c:v>1.6478850865038219</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>1.5946765151252094</c:v>
+                  <c:v>1.6575012440582253</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>1.6192211173831399</c:v>
+                  <c:v>1.682228506340977</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3290,34 +3287,34 @@
       <c r="D3" s="54"/>
       <c r="E3" s="127">
         <f>SUM(E4:E10006)</f>
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="F3" s="55">
         <f>SUM(F4:F10006)</f>
-        <v>246</v>
+        <v>256</v>
       </c>
       <c r="G3" s="55">
         <f>SUM(G4:G10006)</f>
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="H3" s="56"/>
       <c r="I3" s="57">
         <f>SUM(I4:I10006)</f>
-        <v>248.16666666666666</v>
+        <v>258.16666666666663</v>
       </c>
       <c r="J3" s="58">
         <f>SUM(J4:J10006)</f>
-        <v>248.16666666666666</v>
+        <v>258.16666666666663</v>
       </c>
       <c r="K3" s="57"/>
       <c r="L3" s="57"/>
       <c r="M3" s="103">
         <f>N3^(1/2)</f>
-        <v>5.4543560573178569</v>
+        <v>5.494947173944845</v>
       </c>
       <c r="N3" s="121">
         <f>SUM(N4:N10006)</f>
-        <v>29.749999999999996</v>
+        <v>30.194444444444439</v>
       </c>
       <c r="O3" s="114"/>
       <c r="P3" s="59"/>
@@ -3586,7 +3583,7 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="150" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B9" s="131" t="s">
         <v>93</v>
@@ -3642,7 +3639,7 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="150" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B10" s="131"/>
       <c r="C10" s="131"/>
@@ -3691,7 +3688,7 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="150" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B11" s="131"/>
       <c r="C11" s="131"/>
@@ -3743,7 +3740,7 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="150" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B12" s="131"/>
       <c r="C12" s="131"/>
@@ -3795,7 +3792,7 @@
     </row>
     <row r="13" spans="1:17" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A13" s="150" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B13" s="131"/>
       <c r="C13" s="131"/>
@@ -3812,7 +3809,7 @@
         <v>5</v>
       </c>
       <c r="H13" s="131" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I13" s="140">
         <f t="shared" si="5"/>
@@ -3849,7 +3846,7 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="150" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B14" s="131" t="s">
         <v>95</v>
@@ -3905,7 +3902,7 @@
     </row>
     <row r="15" spans="1:17" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A15" s="150" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B15" s="131"/>
       <c r="C15" s="131"/>
@@ -3922,7 +3919,7 @@
         <v>9</v>
       </c>
       <c r="H15" s="151" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I15" s="140">
         <f t="shared" si="5"/>
@@ -4011,12 +4008,12 @@
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="150" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B17" s="131"/>
       <c r="C17" s="131"/>
       <c r="D17" s="131" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E17" s="139">
         <v>3</v>
@@ -4060,7 +4057,7 @@
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="150" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B18" s="131"/>
       <c r="C18" s="131"/>
@@ -4112,12 +4109,12 @@
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="150" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B19" s="131"/>
       <c r="C19" s="131"/>
       <c r="D19" s="131" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E19" s="139">
         <v>3</v>
@@ -4161,26 +4158,30 @@
     </row>
     <row r="20" spans="1:17" ht="28.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="150" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B20" s="131"/>
       <c r="C20" s="131"/>
       <c r="D20" s="131" t="s">
         <v>111</v>
       </c>
-      <c r="E20" s="139"/>
-      <c r="F20" s="139"/>
-      <c r="G20" s="139"/>
-      <c r="H20" s="131" t="s">
-        <v>139</v>
-      </c>
-      <c r="I20" s="140" t="str">
+      <c r="E20" s="139">
+        <v>8</v>
+      </c>
+      <c r="F20" s="139">
+        <v>10</v>
+      </c>
+      <c r="G20" s="139">
+        <v>12</v>
+      </c>
+      <c r="H20" s="131"/>
+      <c r="I20" s="140">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-      <c r="J20" s="141" t="str">
+        <v>10</v>
+      </c>
+      <c r="J20" s="141">
         <f t="shared" si="0"/>
-        <v/>
+        <v>10</v>
       </c>
       <c r="K20" s="142">
         <v>99.73</v>
@@ -4189,17 +4190,17 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="M20" s="144" t="str">
+      <c r="M20" s="144">
         <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="N20" s="145" t="str">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="N20" s="145">
         <f t="shared" si="3"/>
-        <v/>
+        <v>0.44444444444444442</v>
       </c>
       <c r="O20" s="146" t="str">
         <f t="shared" si="4"/>
-        <v/>
+        <v>L</v>
       </c>
       <c r="P20" s="117"/>
       <c r="Q20" s="118" t="str">
@@ -4209,7 +4210,7 @@
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="150" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B21" s="131" t="s">
         <v>92</v>
@@ -4265,7 +4266,7 @@
     </row>
     <row r="22" spans="1:17" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A22" s="150" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B22" s="131"/>
       <c r="C22" s="131"/>
@@ -4317,7 +4318,7 @@
     </row>
     <row r="23" spans="1:17" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A23" s="150" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B23" s="147" t="s">
         <v>121</v>
@@ -4373,7 +4374,7 @@
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="150" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B24" s="131"/>
       <c r="C24" s="131"/>
@@ -4425,7 +4426,7 @@
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="150" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B25" s="131"/>
       <c r="C25" s="131" t="s">
@@ -4479,7 +4480,7 @@
     </row>
     <row r="26" spans="1:17" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A26" s="150" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B26" s="131" t="s">
         <v>125</v>
@@ -4535,7 +4536,7 @@
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="150" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B27" s="131"/>
       <c r="C27" s="131"/>
@@ -4587,7 +4588,7 @@
     </row>
     <row r="28" spans="1:17" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A28" s="150" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B28" s="131"/>
       <c r="C28" s="148" t="s">
@@ -4641,7 +4642,7 @@
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="150" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B29" s="131"/>
       <c r="C29" s="131"/>
@@ -4693,7 +4694,7 @@
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="150" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B30" s="131"/>
       <c r="C30" s="131"/>
@@ -4745,7 +4746,7 @@
     </row>
     <row r="31" spans="1:17" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A31" s="150" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B31" s="147" t="s">
         <v>126</v>
@@ -4801,7 +4802,7 @@
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="150" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B32" s="147"/>
       <c r="C32" s="131"/>
@@ -4850,7 +4851,7 @@
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="150" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B33" s="147"/>
       <c r="C33" s="131" t="s">
@@ -4901,7 +4902,7 @@
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="150" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B34" s="131"/>
       <c r="C34" s="131"/>
@@ -4953,12 +4954,12 @@
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="150" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B35" s="131"/>
       <c r="C35" s="131"/>
       <c r="D35" s="131" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E35" s="139">
         <v>15</v>
@@ -5005,11 +5006,11 @@
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="150" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B36" s="131"/>
       <c r="D36" s="51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E36" s="139">
         <v>2</v>
@@ -15561,19 +15562,19 @@
       </c>
       <c r="B4" s="23">
         <f>IF((Spezifikation!J3-(2*Spezifikation!M3))&lt;0,"NV",(Spezifikation!J3-(2*Spezifikation!M3)))</f>
-        <v>237.25795455203095</v>
+        <v>247.17677231877693</v>
       </c>
       <c r="C4" s="18">
         <f>IF(B4="NV",C5,B4/Einstellungen!$B$53)</f>
-        <v>29.657244319003869</v>
+        <v>30.897096539847116</v>
       </c>
       <c r="D4" s="18">
         <f>IF(B4="NV",D5,B4/Einstellungen!$B$54)</f>
-        <v>1.4828622159501934</v>
+        <v>1.5448548269923559</v>
       </c>
       <c r="E4" s="6">
         <f>IF(B4="NV",E5,B4/Einstellungen!$B$55)</f>
-        <v>0.12357185132918279</v>
+        <v>0.12873790224936299</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -15582,19 +15583,19 @@
       </c>
       <c r="B5" s="23">
         <f>IF((Spezifikation!J3-(1.28*Spezifikation!M3))&lt;0,"NV",(Spezifikation!J3-(1.28*Spezifikation!M3)))</f>
-        <v>241.1850909132998</v>
+        <v>251.13313428401722</v>
       </c>
       <c r="C5" s="18">
         <f>IF(B5="NV",C6,B5/Einstellungen!$B$53)</f>
-        <v>30.148136364162475</v>
+        <v>31.391641785502152</v>
       </c>
       <c r="D5" s="18">
         <f>IF(B5="NV",D6,B5/Einstellungen!$B$54)</f>
-        <v>1.5074068182081237</v>
+        <v>1.5695820892751076</v>
       </c>
       <c r="E5" s="6">
         <f>IF(B5="NV",E6,B5/Einstellungen!$B$55)</f>
-        <v>0.12561723485067697</v>
+        <v>0.13079850743959229</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -15603,19 +15604,19 @@
       </c>
       <c r="B6" s="18">
         <f>IF((Spezifikation!J3-(1*Spezifikation!M3))&lt;0,"NV",(Spezifikation!J3-(1*Spezifikation!M3)))</f>
-        <v>242.7123106093488</v>
+        <v>252.67171949272179</v>
       </c>
       <c r="C6" s="18">
         <f>IF(B6="NV",C7,B6/Einstellungen!$B$53)</f>
-        <v>30.339038826168601</v>
+        <v>31.583964936590224</v>
       </c>
       <c r="D6" s="18">
         <f>IF(B6="NV",D7,B6/Einstellungen!$B$54)</f>
-        <v>1.51695194130843</v>
+        <v>1.5791982468295112</v>
       </c>
       <c r="E6" s="6">
         <f>IF(B6="NV",E7,B6/Einstellungen!$B$55)</f>
-        <v>0.12641266177570251</v>
+        <v>0.13159985390245926</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -15624,19 +15625,19 @@
       </c>
       <c r="B7" s="18">
         <f>IF((Spezifikation!J3-(0.84*Spezifikation!M3))&lt;0,"NV",(Spezifikation!J3-(0.84*Spezifikation!M3)))</f>
-        <v>243.58500757851965</v>
+        <v>253.55091104055296</v>
       </c>
       <c r="C7" s="18">
         <f>IF(B7="NV",C8,B7/Einstellungen!$B$53)</f>
-        <v>30.448125947314956</v>
+        <v>31.69386388006912</v>
       </c>
       <c r="D7" s="18">
         <f>IF(B7="NV",D8,B7/Einstellungen!$B$54)</f>
-        <v>1.5224062973657477</v>
+        <v>1.5846931940034561</v>
       </c>
       <c r="E7" s="6">
         <f>IF(B7="NV",E8,B7/Einstellungen!$B$55)</f>
-        <v>0.12686719144714564</v>
+        <v>0.13205776616695467</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -15645,19 +15646,19 @@
       </c>
       <c r="B8" s="22">
         <f>IF((Spezifikation!J3-(0.67*Spezifikation!M3))&lt;0,"NV",(Spezifikation!J3-(0.67*Spezifikation!M3)))</f>
-        <v>244.51224810826369</v>
+        <v>254.48505206012359</v>
       </c>
       <c r="C8" s="22">
         <f>IF(B8="NV",C9,B8/Einstellungen!$B$53)</f>
-        <v>30.564031013532961</v>
+        <v>31.810631507515449</v>
       </c>
       <c r="D8" s="22">
         <f>IF(B8="NV",D9,B8/Einstellungen!$B$54)</f>
-        <v>1.528201550676648</v>
+        <v>1.5905315753757725</v>
       </c>
       <c r="E8" s="22">
         <f>IF(B8="NV",E9,B8/Einstellungen!$B$55)</f>
-        <v>0.127350129223054</v>
+        <v>0.13254429794798103</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -15666,19 +15667,19 @@
       </c>
       <c r="B9" s="18">
         <f>IF((Spezifikation!J3-(0.52*Spezifikation!M3))&lt;0,"NV",(Spezifikation!J3-(0.52*Spezifikation!M3)))</f>
-        <v>245.33040151686137</v>
+        <v>255.3092941362153</v>
       </c>
       <c r="C9" s="18">
         <f>IF(B9="NV",C10,B9/Einstellungen!$B$53)</f>
-        <v>30.666300189607671</v>
+        <v>31.913661767026912</v>
       </c>
       <c r="D9" s="18">
         <f>IF(B9="NV",D10,B9/Einstellungen!$B$54)</f>
-        <v>1.5333150094803836</v>
+        <v>1.5956830883513455</v>
       </c>
       <c r="E9" s="6">
         <f>IF(B9="NV",E10,B9/Einstellungen!$B$55)</f>
-        <v>0.12777625079003196</v>
+        <v>0.13297359069594547</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -15687,19 +15688,19 @@
       </c>
       <c r="B10" s="18">
         <f>IF((Spezifikation!J3-(0.25*Spezifikation!M3))&lt;0,"NV",(Spezifikation!J3-(0.25*Spezifikation!M3)))</f>
-        <v>246.80307765233718</v>
+        <v>256.79292987318041</v>
       </c>
       <c r="C10" s="18">
         <f>IF(B10="NV",C11,B10/Einstellungen!$B$53)</f>
-        <v>30.850384706542147</v>
+        <v>32.099116234147552</v>
       </c>
       <c r="D10" s="18">
         <f>IF(B10="NV",D11,B10/Einstellungen!$B$54)</f>
-        <v>1.5425192353271073</v>
+        <v>1.6049558117073777</v>
       </c>
       <c r="E10" s="6">
         <f>IF(B10="NV",E11,B10/Einstellungen!$B$55)</f>
-        <v>0.12854326961059229</v>
+        <v>0.13374631764228145</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -15708,19 +15709,19 @@
       </c>
       <c r="B11" s="22">
         <f>Spezifikation!J3</f>
-        <v>248.16666666666666</v>
+        <v>258.16666666666663</v>
       </c>
       <c r="C11" s="22">
         <f>B11/Einstellungen!B53</f>
-        <v>31.020833333333332</v>
+        <v>32.270833333333329</v>
       </c>
       <c r="D11" s="22">
         <f>B11/Einstellungen!B54</f>
-        <v>1.5510416666666667</v>
+        <v>1.6135416666666664</v>
       </c>
       <c r="E11" s="135">
         <f>B11/Einstellungen!B55</f>
-        <v>0.12925347222222222</v>
+        <v>0.13446180555555554</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -15729,19 +15730,19 @@
       </c>
       <c r="B12" s="18">
         <f>Spezifikation!J3+(0.25*Spezifikation!M3)</f>
-        <v>249.53025568099613</v>
+        <v>259.54040346015285</v>
       </c>
       <c r="C12" s="18">
         <f>B12/Einstellungen!B53</f>
-        <v>31.191281960124517</v>
+        <v>32.442550432519106</v>
       </c>
       <c r="D12" s="18">
         <f>B12/Einstellungen!B54</f>
-        <v>1.5595640980062258</v>
+        <v>1.6221275216259552</v>
       </c>
       <c r="E12" s="6">
         <f>B12/Einstellungen!B55</f>
-        <v>0.12996367483385216</v>
+        <v>0.13517729346882962</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -15750,19 +15751,19 @@
       </c>
       <c r="B13" s="18">
         <f>Spezifikation!J3+(0.52*Spezifikation!M3)</f>
-        <v>251.00293181647194</v>
+        <v>261.02403919711793</v>
       </c>
       <c r="C13" s="18">
         <f>B13/Einstellungen!B53</f>
-        <v>31.375366477058993</v>
+        <v>32.628004899639741</v>
       </c>
       <c r="D13" s="18">
         <f>B13/Einstellungen!B54</f>
-        <v>1.5687683238529497</v>
+        <v>1.6314002449819871</v>
       </c>
       <c r="E13" s="6">
         <f>B13/Einstellungen!B55</f>
-        <v>0.13073069365441248</v>
+        <v>0.1359500204151656</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -15771,19 +15772,19 @@
       </c>
       <c r="B14" s="22">
         <f>Spezifikation!J3+(0.67*Spezifikation!M3)</f>
-        <v>251.82108522506962</v>
+        <v>261.84828127320969</v>
       </c>
       <c r="C14" s="22">
         <f>B14/Einstellungen!B53</f>
-        <v>31.477635653133703</v>
+        <v>32.731035159151212</v>
       </c>
       <c r="D14" s="22">
         <f>B14/Einstellungen!B54</f>
-        <v>1.5738817826566851</v>
+        <v>1.6365517579575606</v>
       </c>
       <c r="E14" s="135">
         <f>B14/Einstellungen!B55</f>
-        <v>0.13115681522139042</v>
+        <v>0.13637931316313004</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -15792,19 +15793,19 @@
       </c>
       <c r="B15" s="18">
         <f>Spezifikation!J3+(0.84*Spezifikation!M3)</f>
-        <v>252.74832575481366</v>
+        <v>262.78242229278032</v>
       </c>
       <c r="C15" s="18">
         <f>B15/Einstellungen!B53</f>
-        <v>31.593540719351708</v>
+        <v>32.847802786597541</v>
       </c>
       <c r="D15" s="18">
         <f>B15/Einstellungen!B54</f>
-        <v>1.5796770359675854</v>
+        <v>1.642390139329877</v>
       </c>
       <c r="E15" s="6">
         <f>B15/Einstellungen!B55</f>
-        <v>0.13163975299729877</v>
+        <v>0.13686584494415641</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -15813,19 +15814,19 @@
       </c>
       <c r="B16" s="18">
         <f>Spezifikation!J3+(1*Spezifikation!M3)</f>
-        <v>253.62102272398451</v>
+        <v>263.66161384061149</v>
       </c>
       <c r="C16" s="18">
         <f>B16/Einstellungen!B53</f>
-        <v>31.702627840498064</v>
+        <v>32.957701730076437</v>
       </c>
       <c r="D16" s="18">
         <f>B16/Einstellungen!B54</f>
-        <v>1.5851313920249033</v>
+        <v>1.6478850865038219</v>
       </c>
       <c r="E16" s="6">
         <f>B16/Einstellungen!B55</f>
-        <v>0.13209428266874193</v>
+        <v>0.13732375720865181</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -15834,19 +15835,19 @@
       </c>
       <c r="B17" s="18">
         <f>Spezifikation!J3+(1.28*Spezifikation!M3)</f>
-        <v>255.14824242003351</v>
+        <v>265.20019904931604</v>
       </c>
       <c r="C17" s="18">
         <f>B17/Einstellungen!B53</f>
-        <v>31.893530302504189</v>
+        <v>33.150024881164505</v>
       </c>
       <c r="D17" s="18">
         <f>B17/Einstellungen!B54</f>
-        <v>1.5946765151252094</v>
+        <v>1.6575012440582253</v>
       </c>
       <c r="E17" s="6">
         <f>B17/Einstellungen!B55</f>
-        <v>0.13288970959376745</v>
+        <v>0.13812510367151878</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.8" thickBot="1" x14ac:dyDescent="0.3">
@@ -15855,19 +15856,19 @@
       </c>
       <c r="B18" s="26">
         <f>Spezifikation!J3+(2*Spezifikation!M3)</f>
-        <v>259.07537878130239</v>
+        <v>269.1565610145563</v>
       </c>
       <c r="C18" s="26">
         <f>B18/Einstellungen!B53</f>
-        <v>32.384422347662799</v>
+        <v>33.644570126819538</v>
       </c>
       <c r="D18" s="26">
         <f>B18/Einstellungen!B54</f>
-        <v>1.6192211173831399</v>
+        <v>1.682228506340977</v>
       </c>
       <c r="E18" s="136">
         <f>B18/Einstellungen!B55</f>
-        <v>0.13493509311526167</v>
+        <v>0.14018570886174808</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16004,19 +16005,19 @@
       </c>
       <c r="C14" s="32">
         <f>Aufwandschätzung!B8</f>
-        <v>244.51224810826369</v>
+        <v>254.48505206012359</v>
       </c>
       <c r="D14" s="32">
         <f>Aufwandschätzung!B11</f>
-        <v>248.16666666666666</v>
+        <v>258.16666666666663</v>
       </c>
       <c r="E14" s="32">
         <f>Aufwandschätzung!B14</f>
-        <v>251.82108522506962</v>
+        <v>261.84828127320969</v>
       </c>
       <c r="F14" s="33">
         <f>Aufwandschätzung!B18</f>
-        <v>259.07537878130239</v>
+        <v>269.1565610145563</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -16025,19 +16026,19 @@
       </c>
       <c r="C15" s="34">
         <f>C14/C6</f>
-        <v>31.754837416657622</v>
+        <v>33.050006761055009</v>
       </c>
       <c r="D15" s="34">
         <f>D14/C6</f>
-        <v>32.229437229437231</v>
+        <v>33.52813852813852</v>
       </c>
       <c r="E15" s="34">
         <f>E14/C6</f>
-        <v>32.704037042216832</v>
+        <v>34.006270295222038</v>
       </c>
       <c r="F15" s="35">
         <f>F14/C6</f>
-        <v>33.64615308848083</v>
+        <v>34.955397534357964</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -16087,19 +16088,19 @@
       </c>
       <c r="C19" s="38">
         <f>(C5*C14)+C16+C17</f>
-        <v>33987.202487048657</v>
+        <v>35373.422236357183</v>
       </c>
       <c r="D19" s="38">
         <f>(C5*D14)+D16+D17</f>
-        <v>34495.166666666664</v>
+        <v>35885.166666666664</v>
       </c>
       <c r="E19" s="38">
         <f>(C5*E14)+E16+E17</f>
-        <v>35003.130846284679</v>
+        <v>36396.911096976146</v>
       </c>
       <c r="F19" s="40">
         <f>(C5*F14)+F16+F17</f>
-        <v>36011.477650601031</v>
+        <v>37412.761981023323</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="53.4" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>